<commit_message>
Ajout collection complète scripts PowerShell maintenance + outils CSV/Python
- Scripts PowerShell avec configuration interne pour NAS
- Documentations détaillées pour chaque script
- Outils CSV : concaténation et traitement GMA
- Analyseurs et correcteurs de doublons Python
- Projet calculateur axe routier complet
</commit_message>
<xml_diff>
--- a/01-PROJECTS/python/projets/rapportMensuelV2/smc-data-extractor/examples/extraction_clean_20251027_141837/Convergences_Ligne_SMC_2025_09-OB.xlsx
+++ b/01-PROJECTS/python/projets/rapportMensuelV2/smc-data-extractor/examples/extraction_clean_20251027_141837/Convergences_Ligne_SMC_2025_09-OB.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\data\20-DEVELOPPEMENT\01-PROJECTS\python\projets\rapportMensuelV2\smc-data-extractor\examples\extraction_clean_20251027_141837\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{BA7935F2-B63A-43CA-BAE4-741FF602B855}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{AD1EA617-C976-493E-BCC0-089DC335DF51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{FA2D740F-38A4-40EF-97A6-154EA4AC1FA9}"/>
   </bookViews>
@@ -623,7 +623,7 @@
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="42">
@@ -981,12 +981,12 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8792243C-F03F-4784-98A8-C009E49142B7}">
   <dimension ref="A1:U33"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="12" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1043,15 +1043,15 @@
         <v>BD</v>
       </c>
       <c r="T1" s="1" t="str">
-        <f>L1</f>
-        <v>LI</v>
+        <f>K1</f>
+        <v>LH</v>
       </c>
       <c r="U1" s="1" t="str">
         <f>M1</f>
         <v>LB</v>
       </c>
     </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
@@ -1092,16 +1092,16 @@
         <f>IF(ISBLANK(J2),"",J2)</f>
         <v/>
       </c>
-      <c r="T2" s="1" t="str">
-        <f>IF(ISBLANK(L2),"",L2)</f>
-        <v/>
+      <c r="T2" s="1">
+        <f>IF(ISBLANK(K2),"",K2)</f>
+        <v>-7.0000000000000007E-2</v>
       </c>
       <c r="U2" s="1" t="str">
         <f>IF(ISBLANK(M2),"",M2)</f>
         <v/>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>13</v>
       </c>
@@ -1148,16 +1148,16 @@
         <f t="shared" ref="S3:S33" si="3">IF(ISBLANK(J3),"",J3)</f>
         <v>-42.79</v>
       </c>
-      <c r="T3" s="1" t="str">
-        <f t="shared" ref="T3:T33" si="4">IF(ISBLANK(L3),"",L3)</f>
-        <v/>
+      <c r="T3" s="1">
+        <f t="shared" ref="T3:T33" si="4">IF(ISBLANK(K3),"",K3)</f>
+        <v>-25.06</v>
       </c>
       <c r="U3" s="1">
         <f t="shared" ref="U3:U33" si="5">IF(ISBLANK(M3),"",M3)</f>
         <v>-25.95</v>
       </c>
     </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>13</v>
       </c>
@@ -1204,16 +1204,16 @@
         <f t="shared" si="3"/>
         <v>-0.54</v>
       </c>
-      <c r="T4" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T4" s="1">
+        <f t="shared" si="4"/>
+        <v>0.06</v>
       </c>
       <c r="U4" s="1">
         <f t="shared" si="5"/>
         <v>-1.2</v>
       </c>
     </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
@@ -1260,16 +1260,16 @@
         <f t="shared" si="3"/>
         <v>-37.46</v>
       </c>
-      <c r="T5" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T5" s="1">
+        <f t="shared" si="4"/>
+        <v>-26.55</v>
       </c>
       <c r="U5" s="1">
         <f t="shared" si="5"/>
         <v>-33.25</v>
       </c>
     </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -1316,16 +1316,16 @@
         <f t="shared" si="3"/>
         <v>-0.77</v>
       </c>
-      <c r="T6" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T6" s="1">
+        <f t="shared" si="4"/>
+        <v>-0.64</v>
       </c>
       <c r="U6" s="1">
         <f t="shared" si="5"/>
         <v>-0.87</v>
       </c>
     </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>13</v>
       </c>
@@ -1372,16 +1372,16 @@
         <f t="shared" si="3"/>
         <v>-34.94</v>
       </c>
-      <c r="T7" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T7" s="1">
+        <f t="shared" si="4"/>
+        <v>-22.03</v>
       </c>
       <c r="U7" s="1">
         <f t="shared" si="5"/>
         <v>-15.25</v>
       </c>
     </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
@@ -1431,7 +1431,7 @@
         <v>0.28999999999999998</v>
       </c>
     </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>13</v>
       </c>
@@ -1478,16 +1478,16 @@
         <f t="shared" si="3"/>
         <v>-54.27</v>
       </c>
-      <c r="T9" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T9" s="1">
+        <f t="shared" si="4"/>
+        <v>-24.04</v>
       </c>
       <c r="U9" s="1">
         <f t="shared" si="5"/>
         <v>-34.6</v>
       </c>
     </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>21</v>
       </c>
@@ -1537,7 +1537,7 @@
         <v>-0.37</v>
       </c>
     </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>21</v>
       </c>
@@ -1584,16 +1584,16 @@
         <f t="shared" si="3"/>
         <v>-16.7</v>
       </c>
-      <c r="T11" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T11" s="1">
+        <f t="shared" si="4"/>
+        <v>-7.94</v>
       </c>
       <c r="U11" s="1">
         <f t="shared" si="5"/>
         <v>-17.579999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>21</v>
       </c>
@@ -1643,7 +1643,7 @@
         <v>-1.3</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
@@ -1690,16 +1690,16 @@
         <f t="shared" si="3"/>
         <v>-11.28</v>
       </c>
-      <c r="T13" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T13" s="1">
+        <f t="shared" si="4"/>
+        <v>-10.64</v>
       </c>
       <c r="U13" s="1">
         <f t="shared" si="5"/>
         <v>-26.46</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>21</v>
       </c>
@@ -1740,16 +1740,16 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="T14" s="1">
-        <f t="shared" si="4"/>
-        <v>-3.3</v>
+      <c r="T14" s="1" t="str">
+        <f t="shared" si="4"/>
+        <v/>
       </c>
       <c r="U14" s="1" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>21</v>
       </c>
@@ -1762,9 +1762,6 @@
       <c r="D15" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E15" s="1">
-        <v>0</v>
-      </c>
       <c r="F15" s="1">
         <v>-38.58</v>
       </c>
@@ -1786,35 +1783,32 @@
       <c r="L15" s="1">
         <v>-31.55</v>
       </c>
-      <c r="M15" s="1">
+      <c r="P15" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="Q15" s="1">
+        <f t="shared" si="1"/>
+        <v>-19.309999999999999</v>
+      </c>
+      <c r="R15" s="1">
+        <f t="shared" si="2"/>
+        <v>-35</v>
+      </c>
+      <c r="S15" s="1">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P15" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Q15" s="1">
-        <f t="shared" si="1"/>
-        <v>-19.309999999999999</v>
-      </c>
-      <c r="R15" s="1">
-        <f t="shared" si="2"/>
-        <v>-35</v>
-      </c>
-      <c r="S15" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
       <c r="T15" s="1">
         <f t="shared" si="4"/>
-        <v>-31.55</v>
-      </c>
-      <c r="U15" s="1">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.2">
+        <v>-19.88</v>
+      </c>
+      <c r="U15" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>21</v>
       </c>
@@ -1863,14 +1857,14 @@
       </c>
       <c r="T16" s="1">
         <f t="shared" si="4"/>
-        <v>-14.99</v>
+        <v>-5.42</v>
       </c>
       <c r="U16" s="1" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>21</v>
       </c>
@@ -1883,9 +1877,6 @@
       <c r="D17" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="E17" s="1">
-        <v>0</v>
-      </c>
       <c r="F17" s="1">
         <v>-21.46</v>
       </c>
@@ -1907,35 +1898,32 @@
       <c r="L17" s="1">
         <v>-47.75</v>
       </c>
-      <c r="M17" s="1">
+      <c r="P17" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="Q17" s="1">
+        <f t="shared" si="1"/>
+        <v>-6.15</v>
+      </c>
+      <c r="R17" s="1">
+        <f t="shared" si="2"/>
+        <v>-12.01</v>
+      </c>
+      <c r="S17" s="1">
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="P17" s="1">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Q17" s="1">
-        <f t="shared" si="1"/>
-        <v>-6.15</v>
-      </c>
-      <c r="R17" s="1">
-        <f t="shared" si="2"/>
-        <v>-12.01</v>
-      </c>
-      <c r="S17" s="1">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
       <c r="T17" s="1">
         <f t="shared" si="4"/>
-        <v>-47.75</v>
-      </c>
-      <c r="U17" s="1">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.2">
+        <v>-16.850000000000001</v>
+      </c>
+      <c r="U17" s="1" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
@@ -1987,14 +1975,14 @@
       </c>
       <c r="T18" s="1">
         <f t="shared" si="4"/>
-        <v>0.23</v>
+        <v>-0.31</v>
       </c>
       <c r="U18" s="1" t="str">
         <f t="shared" si="5"/>
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>26</v>
       </c>
@@ -2052,14 +2040,14 @@
       </c>
       <c r="T19" s="1">
         <f t="shared" si="4"/>
-        <v>-36.57</v>
+        <v>-29.95</v>
       </c>
       <c r="U19" s="1">
         <f t="shared" si="5"/>
         <v>-2.87</v>
       </c>
     </row>
-    <row r="20" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>26</v>
       </c>
@@ -2117,14 +2105,14 @@
       </c>
       <c r="T20" s="1">
         <f t="shared" si="4"/>
-        <v>-0.08</v>
+        <v>-0.87</v>
       </c>
       <c r="U20" s="1">
         <f t="shared" si="5"/>
         <v>-0.67</v>
       </c>
     </row>
-    <row r="21" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>26</v>
       </c>
@@ -2182,14 +2170,14 @@
       </c>
       <c r="T21" s="1">
         <f t="shared" si="4"/>
-        <v>-59.99</v>
+        <v>-31.02</v>
       </c>
       <c r="U21" s="1">
         <f t="shared" si="5"/>
         <v>-1.44</v>
       </c>
     </row>
-    <row r="22" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>26</v>
       </c>
@@ -2247,14 +2235,14 @@
       </c>
       <c r="T22" s="1">
         <f t="shared" si="4"/>
-        <v>0.02</v>
+        <v>0.49</v>
       </c>
       <c r="U22" s="1">
         <f t="shared" si="5"/>
         <v>-1.34</v>
       </c>
     </row>
-    <row r="23" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>26</v>
       </c>
@@ -2312,14 +2300,14 @@
       </c>
       <c r="T23" s="1">
         <f t="shared" si="4"/>
-        <v>-63.08</v>
+        <v>-19.809999999999999</v>
       </c>
       <c r="U23" s="1">
         <f t="shared" si="5"/>
         <v>-2.75</v>
       </c>
     </row>
-    <row r="24" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>26</v>
       </c>
@@ -2357,16 +2345,16 @@
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="T24" s="1" t="str">
-        <f t="shared" si="4"/>
+      <c r="T24" s="1">
+        <f t="shared" si="4"/>
+        <v>-1.25</v>
+      </c>
+      <c r="U24" s="1" t="str">
+        <f t="shared" si="5"/>
         <v/>
       </c>
-      <c r="U24" s="1" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.2">
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>26</v>
       </c>
@@ -2424,14 +2412,14 @@
       </c>
       <c r="T25" s="1">
         <f t="shared" si="4"/>
-        <v>-28.51</v>
+        <v>-10.75</v>
       </c>
       <c r="U25" s="1">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>31</v>
       </c>
@@ -2478,16 +2466,16 @@
         <f t="shared" si="3"/>
         <v>-4.18</v>
       </c>
-      <c r="T26" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T26" s="1">
+        <f t="shared" si="4"/>
+        <v>-0.46</v>
       </c>
       <c r="U26" s="1">
         <f t="shared" si="5"/>
         <v>-2.11</v>
       </c>
     </row>
-    <row r="27" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>31</v>
       </c>
@@ -2534,16 +2522,16 @@
         <f t="shared" si="3"/>
         <v>-10.09</v>
       </c>
-      <c r="T27" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T27" s="1">
+        <f t="shared" si="4"/>
+        <v>-4.4400000000000004</v>
       </c>
       <c r="U27" s="1">
         <f t="shared" si="5"/>
         <v>-6.98</v>
       </c>
     </row>
-    <row r="28" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>31</v>
       </c>
@@ -2593,7 +2581,7 @@
         <v>-0.33</v>
       </c>
     </row>
-    <row r="29" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>31</v>
       </c>
@@ -2640,16 +2628,16 @@
         <f t="shared" si="3"/>
         <v>-5.14</v>
       </c>
-      <c r="T29" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T29" s="1">
+        <f t="shared" si="4"/>
+        <v>-4.18</v>
       </c>
       <c r="U29" s="1">
         <f t="shared" si="5"/>
         <v>-7.33</v>
       </c>
     </row>
-    <row r="30" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>34</v>
       </c>
@@ -2696,16 +2684,16 @@
         <f t="shared" si="3"/>
         <v>-1.98</v>
       </c>
-      <c r="T30" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T30" s="1">
+        <f t="shared" si="4"/>
+        <v>-0.78</v>
       </c>
       <c r="U30" s="1">
         <f t="shared" si="5"/>
         <v>-0.72</v>
       </c>
     </row>
-    <row r="31" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>34</v>
       </c>
@@ -2752,16 +2740,16 @@
         <f t="shared" si="3"/>
         <v>-2.93</v>
       </c>
-      <c r="T31" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T31" s="1">
+        <f t="shared" si="4"/>
+        <v>-1.67</v>
       </c>
       <c r="U31" s="1">
         <f t="shared" si="5"/>
         <v>-1.52</v>
       </c>
     </row>
-    <row r="32" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>34</v>
       </c>
@@ -2808,16 +2796,16 @@
         <f t="shared" si="3"/>
         <v>-4.29</v>
       </c>
-      <c r="T32" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T32" s="1">
+        <f t="shared" si="4"/>
+        <v>-0.28000000000000003</v>
       </c>
       <c r="U32" s="1">
         <f t="shared" si="5"/>
         <v>-1.04</v>
       </c>
     </row>
-    <row r="33" spans="1:21" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>34</v>
       </c>
@@ -2864,9 +2852,9 @@
         <f t="shared" si="3"/>
         <v>-15.98</v>
       </c>
-      <c r="T33" s="1" t="str">
-        <f t="shared" si="4"/>
-        <v/>
+      <c r="T33" s="1">
+        <f t="shared" si="4"/>
+        <v>-24.39</v>
       </c>
       <c r="U33" s="1">
         <f t="shared" si="5"/>

</xml_diff>